<commit_message>
Add FP detection (unrealized attack path analysis), reorganize and extract data from the asset table, and consolidate redundant data streams
</commit_message>
<xml_diff>
--- a/docs/资产清单_v3_可导入.xlsx
+++ b/docs/资产清单_v3_可导入.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRIDE映射表" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信任边界表" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="威胁主体表" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系统数据流表" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'接口资产'!$A$1:$G$83</definedName>
@@ -23,9 +24,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'数据资产'!$A$1:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'域属性表'!$A$1:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'功能资产'!$A$1:$C$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'支持资产'!$A$1:$C$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'支持资产'!$A$1:$E$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'信任边界表'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'威胁主体表'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'系统数据流表'!$A$1:$F$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +53,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +125,11 @@
         <fgColor rgb="FFB91C1C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -150,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -189,6 +196,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3626,6 +3636,1838 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>数据流编号</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>产生者</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>用户</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>数据流类型</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>目标功能</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SDF01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>电子围栏、航线、备降点信息</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SDF02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>起飞、悬停、恢复任务、备降、上下电、低压配电盒通道开关及复位、电源变换器复位等控制指令</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SDF03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>飞行机组语音</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SDF04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>飞机运行状态</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SDF05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>飞机告警信息</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SDF06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>RCS</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>音视频数据</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SDF07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>电子围栏、航线、备降点信息</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SDF08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>起飞、悬停、恢复任务、备降、上下电、低压配电盒通道开关及复位、电源变换器复位等控制指令</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SDF09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>飞机运行状态</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>SDF10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>飞机告警信息</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SDF11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>AVCS</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>乘客语音</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>SDF12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>AVCS</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>舱内摄像头视频流</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SDF13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>AVCS</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>下视摄像头视频流</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>SDF14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>AVCS</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>飞行机组语音</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SDF15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DAAS</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>DLS</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>叠加探测信息的视频流</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>SDF16</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>DAAS</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>障碍物类型、距离等状态</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>SDF17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DAAS</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>障碍物类型、距离等告警；刹停告警建议</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>F13</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>SDF18</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>DAAS</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>姿态角、飞行速度等数据</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>SDF19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>转速等状态信息</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>SDF20</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>温度、电压、电流等状态信息</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>F1,F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>SDF21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>转速、温度、电压、电流、故障代码等告警信息</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>SDF22</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>转速控制指令</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>SDF23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>电源变换器、低压配电盒、应急配电盒、应急电池状态信息</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>SDF24</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>电源变换器、低压配电盒、应急配电盒、应急电池告警信息</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>F2,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SDF25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>复位/通道通断指令</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>F2,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>SDF26</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>HVDS</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>高压配电盒状态信息</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SDF27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>HVDS</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>高压配电盒告警信息</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>SDF28</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>HVDS</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>空地状态、电机电压、动力电池电压电流值等信息</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>F1,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>SDF29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>PACKS</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>电池电压、电流、温度等状态信息</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F3,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>SDF30</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>PACKS</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>电池电压、电流、温度等告警信息</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F7,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>SDF31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>PACKS</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>高压上下电指令</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F3,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>SDF32</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>PACKS</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>航空器空地状态、高压配电盒支路继电器状态</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>F1,F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>SDF33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>NAVS</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>导航计算机、卫星接收机、卫星天线、三轴陀螺、三轴加速度计等状态信息</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>SDF34</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>NAVS</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>航向、姿态、速度、加速度、位置等数据信息</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>SDF35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>NAVS</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>航向、姿态、速度、加速度、GNSS位置等告警信息</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>SDF36</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>NAVS</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>RTCM纠偏数据</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>SDF37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>状态信息</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>SDF38</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>告警信息</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>SDF39</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>开伞指令</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>F5,F2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>SDF40</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>加解锁指令</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>SDF41</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>导航数据</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>SDF42</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>备降点数据</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>SDF43</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>电子围栏数据</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>SDF44</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>应急降落微调指令数据</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>SDF45</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>转速控制指令</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>F1,F2,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>SDF46</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>内外环控制量，当前飞行状态及模式</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>F2,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>SDF47</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>飞行包线告警信息，电子围栏告警信息</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>SDF48</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>导航数据</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>F3,F4,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>SDF49</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>探测与避让系统数据</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>F3,F7,F13</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>SDF50</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>飞行航线数据</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>SDF51</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>动力电池电量、功率数据</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>F1,F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>SDF52</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>待飞时间和待飞航程，剩余续航时间和续航里程</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>SDF53</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>当前飞行状态</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>SDF54</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>IMS</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>避让告警信息</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>F2,F3,F5,F7,F13</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>SDF55</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>FMS</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>FCS</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>制导指令</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>F2,F3,F7</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>以下是样例，请勿填写此行以下内容</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr"/>
+      <c r="C57" s="3" t="inlineStr"/>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F57"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"CMD,CONFIG,STATE,DATA,LOAD,ALERT,SENSOR"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5594,12 +7436,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5618,6 +7462,16 @@
           <t>交联接口</t>
         </is>
       </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>安全域</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>关键性</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5631,6 +7485,16 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -5644,6 +7508,16 @@
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5657,6 +7531,16 @@
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -5670,6 +7554,16 @@
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5683,6 +7577,16 @@
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -5696,6 +7600,16 @@
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -5709,6 +7623,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -5722,6 +7646,16 @@
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -5735,6 +7669,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -5748,6 +7692,16 @@
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5761,6 +7715,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -5774,6 +7738,16 @@
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5787,6 +7761,16 @@
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -5800,6 +7784,16 @@
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5813,6 +7807,16 @@
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -5826,6 +7830,16 @@
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5839,6 +7853,16 @@
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -5852,6 +7876,16 @@
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5865,6 +7899,16 @@
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -5878,6 +7922,16 @@
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5891,6 +7945,16 @@
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -5904,6 +7968,16 @@
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5913,9 +7987,19 @@
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C24"/>
+  <autoFilter ref="A1:E24"/>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Internal,External,DMZ,Shared"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>